<commit_message>
Test: Record Sammi's SPM-37 test run
TC01-TC11 pass; TC12 stays blocked until SPM-32 is built.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-37_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-37_Test_Cases.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" tabRatio="600" firstSheet="2" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TC01" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="TC02" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="TC03" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TC04" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TC05" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="TC06" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="TC07" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="TC08" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="TC09" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="TC10" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="TC11" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="TC12" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC01" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC02" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC03" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC04" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC05" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC06" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC07" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC08" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC09" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC10" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC11" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC12" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -39,6 +39,7 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
       <color theme="1"/>
       <sz val="10"/>
@@ -46,21 +47,25 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <color theme="1"/>
       <sz val="10"/>
       <scheme val="minor"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <color rgb="FF1155CC"/>
       <sz val="10"/>
       <u val="single"/>
@@ -203,6 +208,10 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -210,10 +219,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -508,67 +513,66 @@
   </cols>
   <sheetData>
     <row r="1" ht="31" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="18" t="inlineStr">
         <is>
           <t>SPM-37: As the assigned Event Coordinator, I want to cancel an event at any stage so it no longer holds arrangements it doesn't need.</t>
         </is>
       </c>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
-      <c r="G1" s="14" t="n"/>
-      <c r="H1" s="14" t="n"/>
-      <c r="I1" s="15" t="n"/>
-    </row>
-    <row r="2"/>
+      <c r="C1" s="16" t="n"/>
+      <c r="D1" s="16" t="n"/>
+      <c r="E1" s="16" t="n"/>
+      <c r="F1" s="16" t="n"/>
+      <c r="G1" s="16" t="n"/>
+      <c r="H1" s="16" t="n"/>
+      <c r="I1" s="17" t="n"/>
+    </row>
     <row r="3" ht="13" customHeight="1">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="C3" s="16" t="inlineStr">
+      <c r="C3" s="18" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D3" s="16" t="inlineStr">
+      <c r="D3" s="18" t="inlineStr">
         <is>
           <t>Linked AC</t>
         </is>
       </c>
-      <c r="E3" s="16" t="inlineStr">
+      <c r="E3" s="18" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F3" s="16" t="inlineStr">
+      <c r="F3" s="18" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="G3" s="16" t="inlineStr">
+      <c r="G3" s="18" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H3" s="16" t="inlineStr">
+      <c r="H3" s="18" t="inlineStr">
         <is>
           <t>Superseded by</t>
         </is>
       </c>
-      <c r="I3" s="16" t="inlineStr">
+      <c r="I3" s="18" t="inlineStr">
         <is>
           <t>Change #</t>
         </is>
@@ -580,38 +584,38 @@
           <t>TC01</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC01</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>The assigned Coordinator cancels a Planning event with a reason, which releases its approved booking, withdraws its pending request at a second venue and releases its equipment</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>AC1, AC3, AC4, AC8</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="F4" s="15" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="G4" s="13" t="inlineStr">
+      <c r="G4" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H4" s="13" t="n"/>
-      <c r="I4" s="13" t="n"/>
+      <c r="H4" s="15" t="n"/>
+      <c r="I4" s="15" t="n"/>
     </row>
     <row r="5" ht="50" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
@@ -619,38 +623,38 @@
           <t>TC02</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC02</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>A cancelled event's pending venue request leaves Venue Staff's Booking Requests list, while another event's stays on it, and Venue Staff are told its approved booking was released</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>AC4, AC3</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="G5" s="13" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H5" s="13" t="n"/>
-      <c r="I5" s="13" t="n"/>
+      <c r="H5" s="15" t="n"/>
+      <c r="I5" s="15" t="n"/>
     </row>
     <row r="6" ht="25" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -658,38 +662,38 @@
           <t>TC03</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC03</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Cancelling an event frees its venue and its reserved equipment for another event on the same dates</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>AC3, AC1</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="G6" s="13" t="inlineStr">
+      <c r="G6" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H6" s="13" t="n"/>
-      <c r="I6" s="13" t="n"/>
+      <c r="H6" s="15" t="n"/>
+      <c r="I6" s="15" t="n"/>
     </row>
     <row r="7" ht="37.5" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
@@ -697,38 +701,38 @@
           <t>TC04</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC04</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Cancelling an event in Safety review closes its pending safety check, so the Safety Officer no longer sees it to review</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>AC6, AC1</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="G7" s="13" t="inlineStr">
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H7" s="13" t="n"/>
-      <c r="I7" s="13" t="n"/>
+      <c r="H7" s="15" t="n"/>
+      <c r="I7" s="15" t="n"/>
     </row>
     <row r="8" ht="25" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -736,38 +740,38 @@
           <t>TC05</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC05</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>Cancelling an event closes its pending change request without applying the date it proposed</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>AC5</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="G8" s="13" t="inlineStr">
+      <c r="G8" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H8" s="13" t="n"/>
-      <c r="I8" s="13" t="n"/>
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="15" t="n"/>
     </row>
     <row r="9" ht="50" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
@@ -775,38 +779,38 @@
           <t>TC06</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC06</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Cancelling a Confirmed event with open registration takes it off Browse Events, and a registered attendee keeps the registration, can no longer withdraw, and can open the event to see why it was cancelled</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>AC7, AC8</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="G9" s="13" t="inlineStr">
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H9" s="13" t="n"/>
-      <c r="I9" s="13" t="n"/>
+      <c r="H9" s="15" t="n"/>
+      <c r="I9" s="15" t="n"/>
     </row>
     <row r="10" ht="37.5" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -814,38 +818,38 @@
           <t>TC07</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC07</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>Keep event leaves an Approved event as it was, and cancelling it with no reason and nothing to release records that no reason was given</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>AC8, AC1</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
         <is>
           <t>Boundary</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="F10" s="15" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="G10" s="13" t="inlineStr">
+      <c r="G10" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H10" s="13" t="n"/>
-      <c r="I10" s="13" t="n"/>
+      <c r="H10" s="15" t="n"/>
+      <c r="I10" s="15" t="n"/>
     </row>
     <row r="11" ht="37.5" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
@@ -853,38 +857,38 @@
           <t>TC08</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC08</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>An event can be cancelled from the earliest stage it has an assigned Coordinator, Under review, and from Postponed</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>Boundary</t>
         </is>
       </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="G11" s="13" t="inlineStr">
+      <c r="G11" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H11" s="13" t="n"/>
-      <c r="I11" s="13" t="n"/>
+      <c r="H11" s="15" t="n"/>
+      <c r="I11" s="15" t="n"/>
     </row>
     <row r="12" ht="25" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -892,38 +896,38 @@
           <t>TC09</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC09</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>A Completed or Rejected event offers its assigned Coordinator no Cancel event button</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="F12" s="15" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="G12" s="13" t="inlineStr">
+      <c r="G12" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H12" s="13" t="n"/>
-      <c r="I12" s="13" t="n"/>
+      <c r="H12" s="15" t="n"/>
+      <c r="I12" s="15" t="n"/>
     </row>
     <row r="13" ht="37.5" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
@@ -931,38 +935,38 @@
           <t>TC10</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC10</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <t>Another Coordinator, the Event Coordinator Lead and the event's Organiser cannot cancel an event, while its assigned Coordinator can</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E13" s="15" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F13" s="13" t="inlineStr">
+      <c r="F13" s="15" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
+      <c r="G13" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H13" s="13" t="n"/>
-      <c r="I13" s="13" t="n"/>
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="15" t="n"/>
     </row>
     <row r="14" ht="25" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -970,38 +974,38 @@
           <t>TC11</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC11</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>A cancelled event offers no action that would change its status or its arrangements</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>AC9</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
+      <c r="F14" s="15" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="G14" s="13" t="inlineStr">
+      <c r="G14" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H14" s="13" t="n"/>
-      <c r="I14" s="13" t="n"/>
+      <c r="H14" s="15" t="n"/>
+      <c r="I14" s="15" t="n"/>
     </row>
     <row r="15" ht="37.5" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
@@ -1009,75 +1013,73 @@
           <t>TC12</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC12</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>After an event is cancelled, its pending change request shows as closed on the change request screen and can no longer be approved or rejected</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>AC5</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="F15" s="15" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="G15" s="13" t="inlineStr">
+      <c r="G15" s="15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H15" s="13" t="n"/>
-      <c r="I15" s="13" t="n"/>
-    </row>
-    <row r="16"/>
-    <row r="17"/>
+      <c r="H15" s="15" t="n"/>
+      <c r="I15" s="15" t="n"/>
+    </row>
     <row r="18" ht="13" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
         </is>
       </c>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="15" t="n"/>
-      <c r="E18" s="16" t="inlineStr">
+      <c r="C18" s="16" t="n"/>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="18" t="inlineStr">
         <is>
           <t>Covered by</t>
         </is>
       </c>
-      <c r="F18" s="15" t="n"/>
+      <c r="F18" s="17" t="n"/>
     </row>
     <row r="19" ht="85" customHeight="1">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>Given an event has not yet been Completed, when the assigned Coordinator cancels it, then the event status changes to Cancelled.</t>
         </is>
       </c>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="C19" s="16" t="n"/>
+      <c r="D19" s="17" t="n"/>
+      <c r="E19" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC01
 SPM-37-TC03
@@ -1087,173 +1089,173 @@
 SPM-37-TC09</t>
         </is>
       </c>
-      <c r="F19" s="15" t="n"/>
+      <c r="F19" s="17" t="n"/>
     </row>
     <row r="20" ht="17.5" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>Only the assigned Event Coordinator can cancel the event.</t>
         </is>
       </c>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="15" t="n"/>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="C20" s="16" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC10</t>
         </is>
       </c>
-      <c r="F20" s="15" t="n"/>
+      <c r="F20" s="17" t="n"/>
     </row>
     <row r="21" ht="44.5" customHeight="1">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>AC3</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>Cancelling an event releases all of its venue bookings, at every venue, and its equipment reservations so they become available for other events.</t>
         </is>
       </c>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="15" t="n"/>
-      <c r="E21" s="13" t="inlineStr">
+      <c r="C21" s="16" t="n"/>
+      <c r="D21" s="17" t="n"/>
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC01
 SPM-37-TC02
 SPM-37-TC03</t>
         </is>
       </c>
-      <c r="F21" s="15" t="n"/>
+      <c r="F21" s="17" t="n"/>
     </row>
     <row r="22" ht="31" customHeight="1">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>AC4</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>Pending venue booking requests for the event are withdrawn and no longer appear for Venue Staff to review.</t>
         </is>
       </c>
-      <c r="C22" s="14" t="n"/>
-      <c r="D22" s="15" t="n"/>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="C22" s="16" t="n"/>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC01
 SPM-37-TC02</t>
         </is>
       </c>
-      <c r="F22" s="15" t="n"/>
+      <c r="F22" s="17" t="n"/>
     </row>
     <row r="23" ht="31" customHeight="1">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>AC5</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>Pending change requests for the event are closed without being applied.</t>
         </is>
       </c>
-      <c r="C23" s="14" t="n"/>
-      <c r="D23" s="15" t="n"/>
-      <c r="E23" s="13" t="inlineStr">
+      <c r="C23" s="16" t="n"/>
+      <c r="D23" s="17" t="n"/>
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC05
 SPM-37-TC12</t>
         </is>
       </c>
-      <c r="F23" s="15" t="n"/>
+      <c r="F23" s="17" t="n"/>
     </row>
     <row r="24" ht="31" customHeight="1">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>AC6</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>A pending Operational Safety Check for the event is closed and no longer appears for the Safety Officer to review.</t>
         </is>
       </c>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="C24" s="16" t="n"/>
+      <c r="D24" s="17" t="n"/>
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC04</t>
         </is>
       </c>
-      <c r="F24" s="15" t="n"/>
+      <c r="F24" s="17" t="n"/>
     </row>
     <row r="25" ht="31" customHeight="1">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>AC7</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>Registration for the event is closed, and the event is no longer shown to Attendees as open for registration.</t>
         </is>
       </c>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="15" t="n"/>
-      <c r="E25" s="13" t="inlineStr">
+      <c r="C25" s="16" t="n"/>
+      <c r="D25" s="17" t="n"/>
+      <c r="E25" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC06</t>
         </is>
       </c>
-      <c r="F25" s="15" t="n"/>
+      <c r="F25" s="17" t="n"/>
     </row>
     <row r="26" ht="44.5" customHeight="1">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>AC8</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>A reason for cancellation can be recorded.</t>
         </is>
       </c>
-      <c r="C26" s="14" t="n"/>
-      <c r="D26" s="15" t="n"/>
-      <c r="E26" s="13" t="inlineStr">
+      <c r="C26" s="16" t="n"/>
+      <c r="D26" s="17" t="n"/>
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC01
 SPM-37-TC06
 SPM-37-TC07</t>
         </is>
       </c>
-      <c r="F26" s="15" t="n"/>
+      <c r="F26" s="17" t="n"/>
     </row>
     <row r="27" ht="17.5" customHeight="1">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>AC9</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>A cancelled event's status cannot be changed to any other status.</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n"/>
-      <c r="D27" s="15" t="n"/>
-      <c r="E27" s="13" t="inlineStr">
+      <c r="C27" s="16" t="n"/>
+      <c r="D27" s="17" t="n"/>
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>SPM-37-TC11</t>
         </is>
       </c>
-      <c r="F27" s="15" t="n"/>
+      <c r="F27" s="17" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="21">
@@ -1303,7 +1305,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
@@ -1420,7 +1422,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -1485,7 +1487,7 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="13" t="n">
         <v>46317</v>
       </c>
     </row>
@@ -1498,6 +1500,85 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>ee7ae56</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="50" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Step 2: The badge reads 'Completed', and the header has no 'Cancel event' button.
+Step 3: The badge reads 'Rejected', and the header has no 'Cancel event' button.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>049dd3c</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1593,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
@@ -1637,7 +1718,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -1704,7 +1785,7 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="13" t="n">
         <v>46317</v>
       </c>
     </row>
@@ -1717,6 +1798,87 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>ee7ae56</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="87.5" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Step 2: The badge reads 'Planning', and the header has no 'Cancel event' button.
+Step 5: The 'Change coordinator' card is shown, and the header has no 'Cancel event' button.
+Step 8: The badge reads 'Planning', and the header has no 'Cancel event' button.
+Step 11: The header has a 'Cancel event' button.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>049dd3c</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1893,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
@@ -1853,7 +2015,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -1920,7 +2082,7 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="13" t="n">
         <v>46317</v>
       </c>
     </row>
@@ -1933,6 +2095,87 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>ee7ae56</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="175" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Step 2: The badge reads 'Cancelled'. A red alert 'This event was cancelled' reads 'The client's product launch was called off.' The header has none of 'Cancel event', 'Confirm event', 'Submit for safety check', 'Edit event information' or 'Record withdrawal'.
+Step 3: 'SPM37 Hall (SPM37-HAL)' has the 'Released' badge and the line 'Reason for release: Event cancelled: The client's product launch was called off.', with no button. A blue alert reads 'A venue cannot be requested for a completed, cancelled or rejected event.'
+Step 4: A blue alert reads 'This event is cancelled — equipment requirements can no longer be changed.' The 'SPM37 Projector' line has the 'Cancelled' badge, and there is no way to add, change or remove equipment.
+Step 7: The badge reads 'Cancelled', and no 'Change coordinator' card is shown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>049dd3c</t>
         </is>
       </c>
     </row>
@@ -1947,7 +2190,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
@@ -2067,7 +2310,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2083,7 +2326,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Step 3: The dialog listed 'Close 1 pending change request'.
 Step 4: The badge reads 'Cancelled', and the 'When' row still reads '21 Dec 2027, 09:00–12:00'.
@@ -2097,7 +2340,7 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="18" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
@@ -2133,7 +2376,7 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="13" t="n">
         <v>46317</v>
       </c>
     </row>
@@ -2146,6 +2389,86 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>ee7ae56</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="50" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Step 3: The dialog listed 'Close 1 pending change request'.
+Step 4: The badge reads 'Cancelled', and the 'When' row still reads '21 Dec 2027, 09:00–12:00'.
+Step 5: Not possible: there is no change request screen until SPM-32 is built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>SPM-32 not built</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>049dd3c</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2483,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
@@ -2285,7 +2608,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2353,7 +2676,7 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="13" t="n">
         <v>46317</v>
       </c>
     </row>
@@ -2366,6 +2689,88 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>ee7ae56</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="337.5" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Step 2: The Overview shows the 'Planning' badge, and the header has a 'Cancel event' button.
+Step 3: A dialog 'Cancel this event?' reads 'SPM37 Harbour Summit will be marked Cancelled. This can't be undone.' Under 'Cancelling will:' it lists, in this order: 'Release SPM37 Hall (SPM37-HAL) on 2 Nov 2027, 09:00–12:00', 'Withdraw the request for SPM37 Studio (SPM37-STU) on 2 Nov 2027, 09:00–12:00', 'Release 2 × SPM37 Projector' and 'Cancel the request for 1 × SPM37 Lectern Mic'. It has an empty 'Reason (optional)' box and the buttons 'Cancel event' and 'Keep event'.
+Step 5: The dialog closes. A green alert reads 'The event has been cancelled. Its venue bookings and equipment have been released.' The badge reads 'Cancelled'. A red alert 'This event was cancelled' reads 'The client has called off the summit after losing its keynote sponsor.' The header no longer has 'Cancel event'.
+Step 6: The 'Booking requests' card lists 'SPM37 Hall (SPM37-HAL)' with a grey 'Released' badge and the line 'Reason for release: Event cancelled: The client has called off the summit after losing its keynote sponsor.', and 'SPM37 Studio (SPM37-STU)' with a grey 'Withdrawn' badge and the line 'Reason for withdrawal: Event cancelled: The client has called off the summit after losing its keynote sponsor.' Neither row has a 'Release booking' or 'Withdraw request' button. A blue alert reads 'A venue cannot be requested for a completed, cancelled or rejected event.'
+Step 7: A blue alert reads 'This event is cancelled — equipment requirements can no longer be changed.' The 'SPM37 Projector' and 'SPM37 Lectern Mic' lines both have the 'Cancelled' badge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>049dd3c</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2785,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
@@ -2500,7 +2905,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2565,7 +2970,7 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="13" t="n">
         <v>46317</v>
       </c>
     </row>
@@ -2578,6 +2983,85 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>ee7ae56</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="125" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Step 4: Exactly one card matches: 'SPM37 Guarded Event', 'SPM37 Studio (SPM37-STU)', with the 'Pending' badge, 'Requested' '14 Dec 2027, 09:00–12:00', and its 'Approve' and 'Reject with a reason' buttons. No card for 'SPM37 Harbour Summit' is on the page.
+Step 5: The Notifications list has a new notification titled 'Venue booking released' for 'SPM37 Harbour Summit', reading 'Daniel Tan released SPM37 Hall (SPM37-HAL) for &lt;reference&gt; SPM37 Harbour Summit on 2 Nov 2027, 09:00–12:00. Reason: Event cancelled: The client has called off the summit after losing its keynote sponsor.' There is no notification about the withdrawn SPM37 Studio request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>049dd3c</t>
         </is>
       </c>
     </row>
@@ -2592,7 +3076,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
@@ -2730,7 +3214,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2800,7 +3284,7 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="13" t="n">
         <v>46317</v>
       </c>
     </row>
@@ -2813,6 +3297,90 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>ee7ae56</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="212.5" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Step 2: The 'SPM37 Projector' line reads '2 total − 0 out of service − 2 reserved elsewhere = 0 available for these dates' and 'Held by SPM37 Blocking Expo (2 units) until 17 Nov.'
+Step 6: The 'Request a venue booking' form opens for SPM37 Hall, with 'Date' 16 Nov 2027, 'Start time' 09:00 and 'End time' 12:00.
+Step 7: The request is not sent. A red alert reads 'SPM37 Hall is already booked for &lt;reference&gt; SPM37 Blocking Expo on 16 Nov 2027, 09:00–12:00.'
+Step 9: The dialog 'Cancel this event?' lists 'Release SPM37 Hall (SPM37-HAL) on 16 Nov 2027, 09:00–12:00' and 'Release 2 × SPM37 Projector'.
+Step 10: The badge reads 'Cancelled'.
+Step 13: A green alert reads 'Booking request sent to Venue Staff.' The cancelled event's booking no longer blocks the Hall.
+Step 16: The 'SPM37 Projector' line reads '2 total − 0 out of service − 0 reserved elsewhere = 2 available for these dates', with no 'Held by' line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>049dd3c</t>
         </is>
       </c>
     </row>
@@ -2827,7 +3395,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
@@ -2954,7 +3522,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3023,7 +3591,7 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="13" t="n">
         <v>46317</v>
       </c>
     </row>
@@ -3036,6 +3604,89 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>ee7ae56</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="112.5" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Step 2: 'SPM37 Safety Pending' is listed, submitted by Daniel Tan.
+Step 5: The badge reads 'Safety review'.
+Step 6: The dialog 'Cancel this event?' lists 'Release SPM37 Hall (SPM37-HAL) on 18 Nov 2027, 09:00–12:00' and 'Close the pending safety check'.
+Step 7: The badge reads 'Cancelled'.
+Step 10: 'SPM37 Safety Pending' is not listed.
+Step 11: The Overview shows the 'Cancelled' badge, and the header has no 'Record safety decision' button.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>049dd3c</t>
         </is>
       </c>
     </row>
@@ -3050,7 +3701,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
@@ -3172,7 +3823,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3239,7 +3890,7 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="13" t="n">
         <v>46317</v>
       </c>
     </row>
@@ -3252,6 +3903,87 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>ee7ae56</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="100" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Step 2: The badge reads 'Confirmed', and the 'When' row reads '23 Nov 2027, 09:00–12:00'.
+Step 3: The dialog 'Cancel this event?' lists 'Close 1 pending change request'.
+Step 4: The badge reads 'Cancelled'. The 'When' row still reads '23 Nov 2027, 09:00–12:00'.
+Step 7: The organiser sees the 'Cancelled' badge, and the 'When' row reads '23 Nov 2027, 09:00–12:00'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>049dd3c</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3998,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
@@ -3403,7 +4135,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3473,7 +4205,7 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="13" t="n">
         <v>46317</v>
       </c>
     </row>
@@ -3486,6 +4218,90 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>ee7ae56</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="162.5" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Step 2: 'SPM37 Open Workshop' is listed with the 'Open' badge.
+Step 5: The 'SPM37 Open Workshop' row has the 'Registered' badge and a 'Withdraw' button.
+Step 9: The dialog 'Cancel this event?' lists 'Close registration: 1 registered, 0 on the waiting list'.
+Step 11: The badge reads 'Cancelled'.
+Step 14: 'SPM37 Open Workshop' is not listed.
+Step 17: The 'SPM37 Open Workshop' row is still listed with the 'Registered' badge, and it has no 'Withdraw' button.
+Step 18: The event opens with the 'Cancelled' badge. A red alert 'This event was cancelled' reads 'The trainer is unavailable and no replacement could be found.' There is no 'Register' or 'Withdraw' button.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>049dd3c</t>
         </is>
       </c>
     </row>
@@ -3500,7 +4316,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
@@ -3621,7 +4437,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3688,7 +4504,7 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="13" t="n">
         <v>46317</v>
       </c>
     </row>
@@ -3701,6 +4517,87 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>ee7ae56</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="137.5" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Step 2: The badge reads 'Approved', and the header has a 'Cancel event' button.
+Step 3: The dialog 'Cancel this event?' reads 'SPM37 Quiet Approval will be marked Cancelled. This can't be undone.' and 'This event has no venue bookings, equipment or registration to release.'
+Step 4: The dialog closes. The badge still reads 'Approved', and no alert is shown.
+Step 6: The dialog closes. A green alert reads 'The event has been cancelled. Its venue bookings and equipment have been released.' The badge reads 'Cancelled'. A red alert 'This event was cancelled' reads 'No reason was recorded.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>049dd3c</t>
         </is>
       </c>
     </row>
@@ -3715,7 +4612,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
@@ -3842,7 +4739,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3911,7 +4808,7 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="13" t="n">
         <v>46317</v>
       </c>
     </row>
@@ -3924,6 +4821,89 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>ee7ae56</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="125" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Step 2: 'SPM37 Early Call' is listed.
+Step 3: The badge reads 'Under review', the alert 'This request is waiting for your review' is shown, and the header has a 'Cancel event' button.
+Step 5: The badge reads 'Cancelled', and the alert 'This request is waiting for your review' is gone.
+Step 6: 'SPM37 Early Call' is not listed.
+Step 7: The badge reads 'Postponed', and the header has a 'Cancel event' button.
+Step 9: The badge reads 'Cancelled'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>049dd3c</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SPM-37: Unblock TC12 now that SPM-32 is merged
Step 5 now uses SPM-32's real screens: the event's Change requests card,
plus a new step 6 for the coordinator's Change Requests page. TC12 is
marked Updated with a v2 note, and the change is listed in DECOMMISSIONED.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-37_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-37_Test_Cases.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" tabRatio="600" firstSheet="2" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC01" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC02" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC03" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC04" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC05" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC06" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC07" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC08" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC09" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC10" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC11" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC12" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TC01" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TC02" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TC03" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TC04" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="TC05" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="TC06" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="TC07" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="TC08" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="TC09" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="TC10" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="TC11" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="TC12" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -182,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -219,6 +219,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -531,6 +534,7 @@
       <c r="H1" s="16" t="n"/>
       <c r="I1" s="17" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="18" t="inlineStr">
         <is>
@@ -1040,12 +1044,14 @@
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="H15" s="15" t="n"/>
       <c r="I15" s="15" t="n"/>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18" ht="13" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
         <is>
@@ -2190,83 +2196,90 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
     <col width="56.81640625" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>v2 (2026-10-28): SPM-32 (Process Event Change Request) is merged, so the block on this case is lifted, as its pre-conditions said it would be. Step 5 is replaced with SPM-32's real screens: the event's 'Change requests' card on its Overview, and a new step 6 for the coordinator's 'Change Requests' page. SPM-32 has no Approve or Reject button on the list; a pending request has a 'Review' link instead, so 'no Approve or Reject button' now reads 'no Review link'. What the case checks (AC5: cancelling closes the event's pending change request) is unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="13" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="17.5" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>SPM-37-TC12</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
+    <row r="4" ht="44.5" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>After an event is cancelled, its pending change request shows as closed on the change request screen and can no longer be approved or rejected</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="179.5" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
+    <row r="5" ht="179.5" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED until Process Event Change Request (SPM-32) is built: there is no screen yet that lists an event's change requests. Until then, record each run as 'Blocked' with Remarks 'SPM-32 not built'. When SPM-32 is merged, replace step 5 and its expected result with SPM-32's real navigation and labels, and mark this case Updated.
-Run `npm run fixtures:spm37` before this case, and again after it.
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Run `npm run fixtures:spm37` before this case, and again after it.
 'SPM37 Change Closed' (21 Dec 2027, 09:00–12:00, Planning, Daniel Tan; organiser Rachel Ng) has one pending change request from Rachel Ng that proposes moving it to 28 Dec 2027, 09:00–12:00.
 Logged out.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="98.5" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
+    <row r="6" ht="98.5" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>1. Log in as daniel.tan@connectsphere.com / password123
 2. Click 'All Events' in the sidebar and open 'SPM37 Change Closed'
 3. Click 'Cancel event'
 4. Click 'Cancel event' in the dialog
-5. Open the event's change requests on the Process Event Change Request screen (SPM-32)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44.5" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+5. On the event's Overview, find the 'Change requests' card
+6. Click 'Change Requests' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44.5" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Coordinator: Daniel Tan | Organiser: Rachel Ng
 Event: SPM37 Change Closed | When: 21 Dec 2027, 09:00–12:00
@@ -2274,59 +2287,60 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="125.5" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+    <row r="8" ht="125.5" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Step 3: The dialog 'Cancel this event?' lists 'Close 1 pending change request'.
 Step 4: The badge reads 'Cancelled', and the 'When' row still reads '21 Dec 2027, 09:00–12:00'.
-Step 5: The change request proposing 28 Dec 2027, 09:00–12:00 is shown as 'Withdrawn' with the note 'Closed because the event was cancelled.' It has no 'Approve' or 'Reject' button, and it is not among the change requests waiting for a decision.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
+Step 5: The card lists one request, 'Change of details', with the badge 'Withdrawn'. Its 'Starts at' row proposes '28 Dec 2027, 09:00' and its 'Ends at' row '28 Dec 2027, 12:00'. It reads 'Closed because the event was cancelled.' It has no 'Review' link.
+Step 6: 'SPM37 Change Closed' is not listed on the Change Requests page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>kayalvizhi24</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="12.5" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+    <row r="10" ht="12.5" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B10" s="12" t="n">
         <v>46316</v>
       </c>
     </row>
-    <row r="10" ht="12.5" customHeight="1"/>
-    <row r="11" ht="13" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="11" ht="12.5" customHeight="1"/>
+    <row r="12" ht="13" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="6" t="n"/>
-    </row>
-    <row r="12" ht="50" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>Step 3: The dialog listed 'Close 1 pending change request'.
 Step 4: The badge reads 'Cancelled', and the 'When' row still reads '21 Dec 2027, 09:00–12:00'.
@@ -2334,79 +2348,80 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="25" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="14" ht="25" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>Blocked</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="12.5" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>SPM-32 not built</t>
         </is>
       </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Kayalvizhi</t>
+          <t>SPM-32 not built</t>
         </is>
       </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B16" s="13" t="n">
-        <v>46317</v>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Kayalvizhi</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="n">
+        <v>46317</v>
+      </c>
+    </row>
+    <row r="18" ht="12.5" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>ee7ae56</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="19" ht="15.75" customHeight="1"/>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n"/>
-    </row>
-    <row r="20" ht="50" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="B20" s="5" t="n"/>
+    </row>
+    <row r="21" ht="50" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Step 3: The dialog listed 'Close 1 pending change request'.
 Step 4: The badge reads 'Cancelled', and the 'When' row still reads '21 Dec 2027, 09:00–12:00'.
@@ -2414,59 +2429,59 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-    </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>SPM-32 not built</t>
+          <t>Blocked</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Sammi</t>
+          <t>SPM-32 not built</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B24" s="13" t="n">
-        <v>46318</v>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
           <t>Commit</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>049dd3c</t>
         </is>

</xml_diff>

<commit_message>
SPM-37: Record the TC12 run (Pass)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-37_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-37_Test_Cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" tabRatio="600" firstSheet="2" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" tabRatio="600" firstSheet="3" activeTab="12" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -182,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -219,9 +219,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -534,7 +531,6 @@
       <c r="H1" s="16" t="n"/>
       <c r="I1" s="17" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="18" t="inlineStr">
         <is>
@@ -1050,8 +1046,6 @@
       <c r="H15" s="15" t="n"/>
       <c r="I15" s="15" t="n"/>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18" ht="13" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
         <is>
@@ -2196,15 +2190,15 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
     <col width="56.81640625" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+    <row r="1" ht="12.5" customHeight="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>v2 (2026-10-28): SPM-32 (Process Event Change Request) is merged, so the block on this case is lifted, as its pre-conditions said it would be. Step 5 is replaced with SPM-32's real screens: the event's 'Change requests' card on its Overview, and a new step 6 for the coordinator's 'Change Requests' page. SPM-32 has no Approve or Reject button on the list; a pending request has a 'Review' link instead, so 'no Approve or Reject button' now reads 'no Review link'. What the case checks (AC5: cancelling closes the event's pending change request) is unchanged.</t>
         </is>
@@ -2242,7 +2236,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="179.5" customHeight="1">
+    <row r="5" ht="72.5" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2406,7 +2400,6 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1"/>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -2484,6 +2477,88 @@
       <c r="B26" s="3" t="inlineStr">
         <is>
           <t>049dd3c</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n"/>
+    </row>
+    <row r="29" ht="131" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>Step 3: The dialog 'Cancel this event?' lists 'Close 1 pending change request'.
+Step 4: The badge reads 'Cancelled', and the 'When' row still reads '21 Dec 2027, 09:00–12:00'.
+Step 5: The card lists one request, 'Change of details', with the badge 'Withdrawn'. Its 'Starts at' row proposes '28 Dec 2027, 09:00' and its 'Ends at' row '28 Dec 2027, 12:00'. It reads 'Closed because the event was cancelled.' It has no 'Review' link.
+Step 6: 'SPM37 Change Closed' is not listed on the Change Requests page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Retesting after SPM-32 was merged to main</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Kayalvizhi</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="n">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>4adf525</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SPM-37: Record Sammi's TC12 run (Pass)
Rerun of TC12 on 28 Oct 2026 after SPM-32 was merged: Pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-37_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-37_Test_Cases.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" tabRatio="600" firstSheet="3" activeTab="12" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TC01" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="TC02" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="TC03" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TC04" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TC05" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="TC06" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="TC07" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="TC08" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="TC09" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="TC10" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="TC11" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="TC12" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC01" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC02" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC03" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC04" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC05" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC06" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC07" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC08" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC09" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC10" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC11" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC12" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -2190,7 +2190,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.81640625" customWidth="1" min="1" max="1"/>
@@ -2480,7 +2480,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
@@ -2559,6 +2558,87 @@
       <c r="B34" s="3" t="inlineStr">
         <is>
           <t>4adf525</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n"/>
+    </row>
+    <row r="37" ht="131" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>Step 3: The dialog 'Cancel this event?' lists 'Close 1 pending change request'.
+Step 4: The badge reads 'Cancelled', and the 'When' row still reads '21 Dec 2027, 09:00–12:00'.
+Step 5: The card lists one request, 'Change of details', with the badge 'Withdrawn'. Its 'Starts at' row proposes '28 Dec 2027, 09:00' and its 'Ends at' row '28 Dec 2027, 12:00'. It reads 'Closed because the event was cancelled.' It has no 'Review' link.
+Step 6: 'SPM37 Change Closed' is not listed on the Change Requests page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="n">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>d632380</t>
         </is>
       </c>
     </row>

</xml_diff>